<commit_message>
Add incremental Excel updates and formation dashboard
</commit_message>
<xml_diff>
--- a/0. data2(TM_교체현황_고장심각도).xlsx
+++ b/0. data2(TM_교체현황_고장심각도).xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chami\Desktop\AI 에이전트 기반 CBM 플랫폼 자체구축\기초 data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seoul Metro\Desktop\2026 AI 에이전트 관련 사업시행\0. 연구동아리 활동보고서\0. DB자료\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3412B6B7-E71D-49D3-9017-011ED0B9EAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E075232F-4486-4C3F-99C1-8FC85EB7680F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="고장심각도분류" sheetId="1" r:id="rId1"/>
-    <sheet name="교체현황_DB" sheetId="2" r:id="rId2"/>
+    <sheet name="교체현황_DB" sheetId="2" r:id="rId1"/>
+    <sheet name="고장심각도분류" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,6 +28,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1413,6 +1416,69 @@
   </cellStyles>
   <dxfs count="35">
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
       </font>
@@ -1484,69 +1550,6 @@
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1561,44 +1564,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FailureSeverityTable" displayName="FailureSeverityTable" ref="A1:H8" dataDxfId="13">
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="고장코드" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="표준고장유형" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="심각도" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="위험점수" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="표시색" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="체크박스/선택 기준" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="대표 키워드" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ReplacementTable" displayName="ReplacementTable" ref="A1:T129" dataDxfId="20">
+  <tableColumns count="20">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="교체ID" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="교체일자" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="편성" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="차호" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="위치" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="취거TM_시리얼" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="취거TM_제작년도" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="취거TM_제조사" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="부착TM_시리얼" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="부착TM_제작년도" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="부착TM_제조사" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="고장유형(선택)" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="고장코드(자동)" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="심각도(자동)" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="위험점수(자동)" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="고장성교체여부(자동)" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="세부 고장내용" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="취거품 상태(선택)" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="취거품 상태/조치비고" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="데이터검토(자동)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ReplacementTable" displayName="ReplacementTable" ref="A1:T129" dataDxfId="34">
-  <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="교체ID" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="교체일자" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="편성" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="차호" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="위치" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="취거TM_시리얼" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="취거TM_제작년도" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="취거TM_제조사" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="부착TM_시리얼" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="부착TM_제작년도" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="부착TM_제조사" dataDxfId="23"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="고장유형(선택)" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="고장코드(자동)" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="심각도(자동)" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="위험점수(자동)" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="고장성교체여부(자동)" dataDxfId="18"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0100-000012000000}" name="세부 고장내용" dataDxfId="17"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="취거품 상태(선택)" dataDxfId="16"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="취거품 상태/조치비고" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="데이터검토(자동)" dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FailureSeverityTable" displayName="FailureSeverityTable" ref="A1:H8" dataDxfId="34">
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="고장코드" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="표준고장유형" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="심각도" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="위험점수" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="표시색" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="체크박스/선택 기준" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="대표 키워드" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="비고" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1752,333 +1755,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="28" style="10" customWidth="1"/>
-    <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="34" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="21" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="4">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4">
-        <v>10</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="4">
-        <v>4</v>
-      </c>
-      <c r="D4" s="4">
-        <v>20</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="4">
-        <v>5</v>
-      </c>
-      <c r="D5" s="4">
-        <v>45</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="4">
-        <v>6</v>
-      </c>
-      <c r="D6" s="4">
-        <v>70</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="4">
-        <v>7</v>
-      </c>
-      <c r="D7" s="4">
-        <v>100</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" s="6" customFormat="1" ht="29" customHeight="1">
-      <c r="A8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4">
-        <v>5</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="3"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="3"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:T129"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="5" width="8" customWidth="1"/>
@@ -2099,7 +1778,7 @@
     <col min="20" max="20" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="28">
+    <row r="1" spans="1:20" ht="30">
       <c r="A1" s="2" t="s">
         <v>67</v>
       </c>
@@ -10366,23 +10045,23 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="N2:N129">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="greaterThanOrEqual">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="24" priority="2" operator="between">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="23" priority="3" operator="between">
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R2:R129">
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="22" priority="4">
       <formula>OR($R2="정비불가",$R2="폐기/불용")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T2:T129">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="21" priority="5">
       <formula>$T2="확인필요"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10409,4 +10088,328 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="28" style="10" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="42" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="21" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3"/>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="4">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="4">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4">
+        <v>45</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="4">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4">
+        <v>70</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="4">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4">
+        <v>100</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" s="6" customFormat="1" ht="29.1" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <v>5</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="3"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="3"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>